<commit_message>
Update Word documentation and Excel feature inventory
</commit_message>
<xml_diff>
--- a/機能一覧.xlsx
+++ b/機能一覧.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\accounting\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CEFCA45-B228-4A26-81F3-41B51BE7B1DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC12ABD1-5980-46A0-8DC6-3D8DEBE093BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{CEA7EC07-4F09-40C1-B1AF-DE05FAF8DEE6}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="183">
   <si>
     <t>機能分類</t>
   </si>
@@ -594,6 +594,13 @@
     <t>エンハンス日</t>
     <rPh sb="5" eb="6">
       <t>ヒ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>もんじゃ会計</t>
+    <rPh sb="4" eb="6">
+      <t>カイケイ</t>
     </rPh>
     <phoneticPr fontId="1"/>
   </si>
@@ -1019,7 +1026,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{750440B3-0B04-4072-80D1-98B6638A41C3}">
-  <dimension ref="A1:G76"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:G77"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="13" style="2" bestFit="1" customWidth="1"/>
@@ -1032,56 +1042,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="2" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F2" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G2" s="4" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="3">
-        <v>46307</v>
-      </c>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>7</v>
@@ -1097,10 +1093,10 @@
         <v>4</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>7</v>
@@ -1113,13 +1109,13 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>7</v>
@@ -1135,10 +1131,10 @@
         <v>12</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>7</v>
@@ -1154,10 +1150,10 @@
         <v>12</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>7</v>
@@ -1173,46 +1169,46 @@
         <v>12</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
+        <v>7</v>
+      </c>
+      <c r="E8" s="3">
+        <v>46307</v>
+      </c>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A9" s="1" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E9" s="3">
-        <v>46307</v>
-      </c>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
+        <v>21</v>
+      </c>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A10" s="1" t="s">
         <v>22</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>7</v>
@@ -1228,10 +1224,10 @@
         <v>22</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>7</v>
@@ -1244,13 +1240,13 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A12" s="1" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>7</v>
@@ -1266,10 +1262,10 @@
         <v>29</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>7</v>
@@ -1282,13 +1278,13 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A14" s="1" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>7</v>
@@ -1304,10 +1300,10 @@
         <v>34</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>7</v>
@@ -1323,10 +1319,10 @@
         <v>34</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>7</v>
@@ -1342,10 +1338,10 @@
         <v>34</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>7</v>
@@ -1361,10 +1357,10 @@
         <v>34</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>7</v>
@@ -1380,10 +1376,10 @@
         <v>34</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>7</v>
@@ -1396,13 +1392,13 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A20" s="1" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>7</v>
@@ -1418,10 +1414,10 @@
         <v>47</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>7</v>
@@ -1437,10 +1433,10 @@
         <v>47</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>7</v>
@@ -1456,10 +1452,10 @@
         <v>47</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>7</v>
@@ -1475,27 +1471,29 @@
         <v>47</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
-      <c r="G24" s="1"/>
+        <v>7</v>
+      </c>
+      <c r="E24" s="3">
+        <v>46307</v>
+      </c>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A25" s="1" t="s">
         <v>47</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>21</v>
@@ -1506,32 +1504,30 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A26" s="1" t="s">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E26" s="3">
-        <v>46307</v>
-      </c>
-      <c r="F26" s="3"/>
-      <c r="G26" s="3"/>
+        <v>21</v>
+      </c>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="1"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A27" s="1" t="s">
         <v>60</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>7</v>
@@ -1547,82 +1543,82 @@
         <v>60</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E28" s="1"/>
-      <c r="F28" s="1"/>
-      <c r="G28" s="1"/>
+        <v>7</v>
+      </c>
+      <c r="E28" s="3">
+        <v>46307</v>
+      </c>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A29" s="1" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E29" s="3">
-        <v>46307</v>
-      </c>
-      <c r="F29" s="3"/>
-      <c r="G29" s="3"/>
+        <v>21</v>
+      </c>
+      <c r="E29" s="1"/>
+      <c r="F29" s="1"/>
+      <c r="G29" s="1"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A30" s="1" t="s">
         <v>67</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E30" s="1"/>
-      <c r="F30" s="1"/>
-      <c r="G30" s="1"/>
+        <v>7</v>
+      </c>
+      <c r="E30" s="3">
+        <v>46307</v>
+      </c>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A31" s="1" t="s">
         <v>67</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E31" s="3">
-        <v>46307</v>
-      </c>
-      <c r="F31" s="3"/>
-      <c r="G31" s="3"/>
+        <v>21</v>
+      </c>
+      <c r="E31" s="1"/>
+      <c r="F31" s="1"/>
+      <c r="G31" s="1"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A32" s="1" t="s">
         <v>67</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D32" s="1" t="s">
         <v>7</v>
@@ -1638,10 +1634,10 @@
         <v>67</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D33" s="1" t="s">
         <v>7</v>
@@ -1657,27 +1653,29 @@
         <v>67</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E34" s="1"/>
-      <c r="F34" s="1"/>
-      <c r="G34" s="1"/>
+        <v>7</v>
+      </c>
+      <c r="E34" s="3">
+        <v>46307</v>
+      </c>
+      <c r="F34" s="3"/>
+      <c r="G34" s="3"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A35" s="1" t="s">
         <v>67</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D35" s="1" t="s">
         <v>21</v>
@@ -1691,10 +1689,10 @@
         <v>67</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D36" s="1" t="s">
         <v>21</v>
@@ -1705,49 +1703,49 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A37" s="1" t="s">
-        <v>84</v>
+        <v>67</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="E37" s="3">
-        <v>46307</v>
-      </c>
-      <c r="F37" s="3"/>
-      <c r="G37" s="3"/>
+        <v>21</v>
+      </c>
+      <c r="E37" s="1"/>
+      <c r="F37" s="1"/>
+      <c r="G37" s="1"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A38" s="1" t="s">
         <v>84</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E38" s="1"/>
-      <c r="F38" s="1"/>
-      <c r="G38" s="1"/>
+        <v>87</v>
+      </c>
+      <c r="E38" s="3">
+        <v>46307</v>
+      </c>
+      <c r="F38" s="3"/>
+      <c r="G38" s="3"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A39" s="1" t="s">
         <v>84</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D39" s="1" t="s">
         <v>21</v>
@@ -1758,32 +1756,30 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A40" s="1" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E40" s="3">
-        <v>46307</v>
-      </c>
-      <c r="F40" s="3"/>
-      <c r="G40" s="3"/>
+        <v>21</v>
+      </c>
+      <c r="E40" s="1"/>
+      <c r="F40" s="1"/>
+      <c r="G40" s="1"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A41" s="1" t="s">
         <v>92</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D41" s="1" t="s">
         <v>7</v>
@@ -1799,10 +1795,10 @@
         <v>92</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D42" s="1" t="s">
         <v>7</v>
@@ -1818,10 +1814,10 @@
         <v>92</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D43" s="1" t="s">
         <v>7</v>
@@ -1837,10 +1833,10 @@
         <v>92</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D44" s="1" t="s">
         <v>7</v>
@@ -1856,10 +1852,10 @@
         <v>92</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D45" s="1" t="s">
         <v>7</v>
@@ -1875,46 +1871,46 @@
         <v>92</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E46" s="1"/>
-      <c r="F46" s="1"/>
-      <c r="G46" s="1"/>
+        <v>7</v>
+      </c>
+      <c r="E46" s="3">
+        <v>46307</v>
+      </c>
+      <c r="F46" s="3"/>
+      <c r="G46" s="3"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A47" s="1" t="s">
-        <v>107</v>
+        <v>92</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E47" s="3">
-        <v>46307</v>
-      </c>
-      <c r="F47" s="3"/>
-      <c r="G47" s="3"/>
+        <v>21</v>
+      </c>
+      <c r="E47" s="1"/>
+      <c r="F47" s="1"/>
+      <c r="G47" s="1"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A48" s="1" t="s">
         <v>107</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D48" s="1" t="s">
         <v>7</v>
@@ -1927,13 +1923,13 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A49" s="1" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="D49" s="1" t="s">
         <v>7</v>
@@ -1949,10 +1945,10 @@
         <v>112</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D50" s="1" t="s">
         <v>7</v>
@@ -1968,10 +1964,10 @@
         <v>112</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D51" s="1" t="s">
         <v>7</v>
@@ -1984,13 +1980,13 @@
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A52" s="1" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="D52" s="1" t="s">
         <v>7</v>
@@ -2003,13 +1999,13 @@
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A53" s="1" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D53" s="1" t="s">
         <v>7</v>
@@ -2025,82 +2021,82 @@
         <v>122</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E54" s="1"/>
-      <c r="F54" s="1"/>
-      <c r="G54" s="1"/>
+        <v>7</v>
+      </c>
+      <c r="E54" s="3">
+        <v>46307</v>
+      </c>
+      <c r="F54" s="3"/>
+      <c r="G54" s="3"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A55" s="1" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E55" s="3">
-        <v>46307</v>
-      </c>
-      <c r="F55" s="3"/>
-      <c r="G55" s="3"/>
+        <v>21</v>
+      </c>
+      <c r="E55" s="1"/>
+      <c r="F55" s="1"/>
+      <c r="G55" s="1"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A56" s="1" t="s">
         <v>119</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E56" s="1"/>
-      <c r="F56" s="1"/>
-      <c r="G56" s="1"/>
+        <v>7</v>
+      </c>
+      <c r="E56" s="3">
+        <v>46307</v>
+      </c>
+      <c r="F56" s="3"/>
+      <c r="G56" s="3"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A57" s="1" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E57" s="3">
-        <v>46307</v>
-      </c>
-      <c r="F57" s="3"/>
-      <c r="G57" s="3"/>
+        <v>21</v>
+      </c>
+      <c r="E57" s="1"/>
+      <c r="F57" s="1"/>
+      <c r="G57" s="1"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A58" s="1" t="s">
         <v>131</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D58" s="1" t="s">
         <v>7</v>
@@ -2116,10 +2112,10 @@
         <v>131</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D59" s="1" t="s">
         <v>7</v>
@@ -2135,46 +2131,46 @@
         <v>131</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E60" s="1"/>
-      <c r="F60" s="1"/>
-      <c r="G60" s="1"/>
+        <v>7</v>
+      </c>
+      <c r="E60" s="3">
+        <v>46307</v>
+      </c>
+      <c r="F60" s="3"/>
+      <c r="G60" s="3"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A61" s="1" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E61" s="3">
-        <v>46307</v>
-      </c>
-      <c r="F61" s="3"/>
-      <c r="G61" s="3"/>
+        <v>21</v>
+      </c>
+      <c r="E61" s="1"/>
+      <c r="F61" s="1"/>
+      <c r="G61" s="1"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A62" s="1" t="s">
         <v>140</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D62" s="1" t="s">
         <v>7</v>
@@ -2187,13 +2183,13 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A63" s="1" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="D63" s="1" t="s">
         <v>7</v>
@@ -2206,13 +2202,13 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A64" s="1" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="D64" s="1" t="s">
         <v>7</v>
@@ -2228,27 +2224,29 @@
         <v>148</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E65" s="1"/>
-      <c r="F65" s="1"/>
-      <c r="G65" s="1"/>
+        <v>7</v>
+      </c>
+      <c r="E65" s="3">
+        <v>46307</v>
+      </c>
+      <c r="F65" s="3"/>
+      <c r="G65" s="3"/>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A66" s="1" t="s">
         <v>148</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D66" s="1" t="s">
         <v>21</v>
@@ -2259,32 +2257,30 @@
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A67" s="1" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E67" s="3">
-        <v>46307</v>
-      </c>
-      <c r="F67" s="3"/>
-      <c r="G67" s="3"/>
+        <v>21</v>
+      </c>
+      <c r="E67" s="1"/>
+      <c r="F67" s="1"/>
+      <c r="G67" s="1"/>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A68" s="1" t="s">
         <v>155</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D68" s="1" t="s">
         <v>7</v>
@@ -2297,13 +2293,13 @@
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A69" s="1" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="D69" s="1" t="s">
         <v>7</v>
@@ -2319,10 +2315,10 @@
         <v>160</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="D70" s="1" t="s">
         <v>7</v>
@@ -2338,10 +2334,10 @@
         <v>160</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="D71" s="1" t="s">
         <v>7</v>
@@ -2357,13 +2353,13 @@
         <v>160</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>87</v>
+        <v>7</v>
       </c>
       <c r="E72" s="3">
         <v>46307</v>
@@ -2373,16 +2369,16 @@
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A73" s="1" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>7</v>
+        <v>87</v>
       </c>
       <c r="E73" s="3">
         <v>46307</v>
@@ -2392,13 +2388,13 @@
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A74" s="1" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="D74" s="1" t="s">
         <v>7</v>
@@ -2411,30 +2407,32 @@
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A75" s="1" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E75" s="1"/>
-      <c r="F75" s="1"/>
-      <c r="G75" s="1"/>
+        <v>7</v>
+      </c>
+      <c r="E75" s="3">
+        <v>46307</v>
+      </c>
+      <c r="F75" s="3"/>
+      <c r="G75" s="3"/>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A76" s="1" t="s">
         <v>175</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D76" s="1" t="s">
         <v>21</v>
@@ -2443,8 +2441,26 @@
       <c r="F76" s="1"/>
       <c r="G76" s="1"/>
     </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A77" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="D77" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E77" s="1"/>
+      <c r="F77" s="1"/>
+      <c r="G77" s="1"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.39370078740157483" bottom="0.39370078740157483" header="0.39370078740157483" footer="0.39370078740157483"/>
+  <pageSetup paperSize="9" scale="47" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>